<commit_message>
Localize case review workbook labels
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.zh.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.zh.xlsx
@@ -945,27 +945,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1100,27 +1100,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1253,27 +1253,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1416,27 +1416,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1564,27 +1564,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1716,37 +1716,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2155,27 +2155,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2317,27 +2317,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -2469,27 +2469,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -2611,27 +2611,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -2780,37 +2780,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3219,27 +3219,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -3388,27 +3388,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -3539,27 +3539,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -3708,37 +3708,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4147,27 +4147,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>policy_direct_answer_special</t>
+          <t>策略请求：直接要答案/代码</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>safe_redirect</t>
+          <t>安全重定向</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -4301,27 +4301,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>policy_direct_answer_special</t>
+          <t>策略请求：直接要答案/代码</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>safe_redirect</t>
+          <t>安全重定向</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -4449,27 +4449,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>policy_direct_answer_special</t>
+          <t>策略请求：直接要答案/代码</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>safe_redirect</t>
+          <t>安全重定向</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -4614,37 +4614,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5053,27 +5053,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -5175,27 +5175,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -5296,27 +5296,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -5427,27 +5427,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -5550,27 +5550,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -5677,27 +5677,27 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -5810,27 +5810,27 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -5937,27 +5937,27 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -6067,27 +6067,27 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -6191,27 +6191,27 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -6331,27 +6331,27 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -6499,27 +6499,27 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -6642,27 +6642,27 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -6784,27 +6784,27 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -6922,27 +6922,27 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -7080,27 +7080,27 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -7220,27 +7220,27 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -7363,27 +7363,27 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -7508,27 +7508,27 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -7660,27 +7660,27 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -7813,27 +7813,27 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -7957,27 +7957,27 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -8144,27 +8144,27 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -8293,27 +8293,27 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -8445,27 +8445,27 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -8595,27 +8595,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -8737,27 +8737,27 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -8912,27 +8912,27 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -9083,27 +9083,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -9244,27 +9244,27 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -9398,27 +9398,27 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -9542,27 +9542,27 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -9702,27 +9702,27 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -9856,27 +9856,27 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -10022,27 +10022,27 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -10171,27 +10171,27 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -10326,27 +10326,27 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -10479,27 +10479,27 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -10642,27 +10642,27 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -10790,27 +10790,27 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -10951,27 +10951,27 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -11113,27 +11113,27 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -11265,27 +11265,27 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -11407,27 +11407,27 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -11585,27 +11585,27 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -11754,27 +11754,27 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -11905,27 +11905,27 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>followup_after_prerequisite_gap</t>
+          <t>基础断层：前置概念缺口后续轮</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4 基础断层</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>prerequisite_repair</t>
+          <t>补前置概念</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -12083,27 +12083,27 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>policy_direct_answer_special</t>
+          <t>策略请求：直接要答案/代码</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>safe_redirect</t>
+          <t>安全重定向</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -12237,27 +12237,27 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>policy_direct_answer_special</t>
+          <t>策略请求：直接要答案/代码</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>safe_redirect</t>
+          <t>安全重定向</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -12385,27 +12385,27 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>policy_direct_answer_special</t>
+          <t>策略请求：直接要答案/代码</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>safe_redirect</t>
+          <t>安全重定向</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -12550,37 +12550,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12989,27 +12989,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -13111,27 +13111,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -13232,27 +13232,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -13363,27 +13363,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -13486,27 +13486,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -13613,27 +13613,27 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -13737,37 +13737,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14176,27 +14176,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -14303,27 +14303,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -14433,27 +14433,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -14557,27 +14557,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>initial</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>initial_question</t>
+          <t>初始提问</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>不适用</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -14697,27 +14697,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -14856,37 +14856,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15295,27 +15295,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -15438,27 +15438,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -15580,27 +15580,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -15718,27 +15718,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -15876,27 +15876,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -16007,37 +16007,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16446,27 +16446,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_correct_short_answer</t>
+          <t>能跟上：短答正确后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 能一直跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>advance</t>
+          <t>推进到下一小步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -16589,27 +16589,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -16734,27 +16734,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -16886,27 +16886,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -17039,27 +17039,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -17174,37 +17174,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17613,27 +17613,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -17800,27 +17800,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -17949,27 +17949,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -18101,27 +18101,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_partial_answer</t>
+          <t>部分跟上：回答不完整后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>clarify</t>
+          <t>澄清当前回答</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -18251,27 +18251,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -18384,37 +18384,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18823,27 +18823,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -18998,27 +18998,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -19169,27 +19169,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -19330,27 +19330,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -19475,37 +19475,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19914,27 +19914,27 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -20058,27 +20058,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>followup_after_wrong_answer</t>
+          <t>跟得吃力：回答错误后续轮</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3 比较难跟上</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -20218,27 +20218,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -20372,27 +20372,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -20538,27 +20538,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>followup</t>
+          <t>后续辅导轮</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>followup_after_code_attempt</t>
+          <t>部分跟上：代码尝试后续轮</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2 勉强/部分跟上</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>micro_step</t>
+          <t>拆成更小一步</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -20678,37 +20678,37 @@
   <autoFilter ref="A2:AH2"/>
   <dataValidations count="11">
     <dataValidation sqref="W3:W7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="X3:X7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Y3:Y7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,partial,no"</formula1>
+      <formula1>"是,部分,否"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,not_applicable"</formula1>
+      <formula1>"是,需修改,否,不适用"</formula1>
     </dataValidation>
     <dataValidation sqref="AA3:AA7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AB3:AB7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,too_strict,too_loose,unclear"</formula1>
+      <formula1>"是,过严,过松,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no"</formula1>
+      <formula1>"是,需修改,否"</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"yes,revise,no,unclear"</formula1>
+      <formula1>"是,需修改,否,不清楚"</formula1>
     </dataValidation>
     <dataValidation sqref="AE3:AE7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"accept,revise,drop,discuss"</formula1>
+      <formula1>"接受,修改,丢弃,讨论"</formula1>
     </dataValidation>
     <dataValidation sqref="AF3:AF7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"none,source_issue,context_mismatch,student_language_artificial,followability_issue,bridge_label_issue,forbidden_content_issue,success_criteria_issue,leakage_boundary_issue,other"</formula1>
+      <formula1>"无,题源问题,上下文不一致,学生话术不像真实学生,跟随状态问题,桥梁标签问题,禁止内容问题,成功标准问题,泄露边界问题,其他"</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid review code" error="Please choose one of the allowed review codes." promptTitle="Structured review" prompt="Use the dropdown value so the review can be summarized." type="list">
-      <formula1>"high,medium,low"</formula1>
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Clarify Chinese review workbook choices
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.zh.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_50_source_and_case_review.zh.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>6. 结构化审核列使用固定英文选项，便于统计：case_decision 填 accept / revise / drop / discuss。</t>
+          <t>6. 结构化审核列使用固定中文选项，统计脚本会映射为英文 canonical values。例如：接受=accept，修改=revise，丢弃=drop，讨论=discuss。</t>
         </is>
       </c>
     </row>
@@ -535,6 +535,13 @@
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>7. 本表是 case/source 复核，不是 AI 回复盲评；此时不评价任何 condition 的回复质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8. context_ai_reply / prior_ai_scaffold 只用于判断学生当前回复是否承接上一轮脚手架，不用于评价该 AI 回复本身好坏。</t>
         </is>
       </c>
     </row>

</xml_diff>